<commit_message>
fix: add ไม่ทราบสถานะ to IT status example in Import_Template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/client/Import_Template.xlsx
+++ b/dist/client/Import_Template.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07D9395-79A3-4D6A-9951-7824F6E2B41D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Template" state="visible" r:id="rId4"/>
+    <sheet name="Template" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -97,9 +106,6 @@
     <t>example@email.com</t>
   </si>
   <si>
-    <t>ดำเนินการแล้ว / ยังไม่ดำเนินการ / ไม่พบบัญชี</t>
-  </si>
-  <si>
     <t>วว/ดด/ปปปป (พ.ศ.)</t>
   </si>
   <si>
@@ -144,30 +150,33 @@
   <si>
     <t>ไม่พบบัญชี</t>
   </si>
+  <si>
+    <t>ดำเนินการแล้ว / ยังไม่ดำเนินการ / ไม่พบบัญชี / ไม่ทราบสถานะ</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Tahoma"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
       <name val="TH Sarabun New"/>
     </font>
     <font>
       <b/>
       <i/>
+      <sz val="14"/>
       <color rgb="FFFF0000"/>
-      <sz val="14"/>
       <name val="TH Sarabun New"/>
     </font>
     <font>
@@ -207,10 +216,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -588,9 +605,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U200"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="3" width="8" customWidth="1"/>
@@ -612,7 +629,7 @@
     <col min="21" max="21" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -677,7 +694,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
@@ -708,31 +725,31 @@
         <v>27</v>
       </c>
       <c r="N2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="P2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="R2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="S2" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="T2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="U2" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -743,57 +760,57 @@
         <v>2599</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="M3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="Q3" s="3"/>
       <c r="R3" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="S3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="T3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="T3" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="U3" s="3"/>
     </row>
-    <row r="4" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -816,7 +833,7 @@
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
     </row>
-    <row r="5" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -839,7 +856,7 @@
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
     </row>
-    <row r="6" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -862,7 +879,7 @@
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
     </row>
-    <row r="7" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -885,7 +902,7 @@
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
     </row>
-    <row r="8" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -908,7 +925,7 @@
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
     </row>
-    <row r="9" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -931,7 +948,7 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
     </row>
-    <row r="10" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -954,7 +971,7 @@
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
     </row>
-    <row r="11" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -977,7 +994,7 @@
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
     </row>
-    <row r="12" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -1000,7 +1017,7 @@
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
     </row>
-    <row r="13" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -1023,7 +1040,7 @@
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
     </row>
-    <row r="14" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1046,7 +1063,7 @@
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
     </row>
-    <row r="15" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -1069,7 +1086,7 @@
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
     </row>
-    <row r="16" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1092,7 +1109,7 @@
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
     </row>
-    <row r="17" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -1115,7 +1132,7 @@
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
     </row>
-    <row r="18" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -1138,7 +1155,7 @@
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
     </row>
-    <row r="19" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1161,7 +1178,7 @@
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
     </row>
-    <row r="20" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1184,7 +1201,7 @@
       <c r="T20" s="3"/>
       <c r="U20" s="3"/>
     </row>
-    <row r="21" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1207,7 +1224,7 @@
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
     </row>
-    <row r="22" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1230,7 +1247,7 @@
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
     </row>
-    <row r="23" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1253,7 +1270,7 @@
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
     </row>
-    <row r="24" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1276,7 +1293,7 @@
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
     </row>
-    <row r="25" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1299,7 +1316,7 @@
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
     </row>
-    <row r="26" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1322,7 +1339,7 @@
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
     </row>
-    <row r="27" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1345,7 +1362,7 @@
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
     </row>
-    <row r="28" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1368,7 +1385,7 @@
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
     </row>
-    <row r="29" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1391,7 +1408,7 @@
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
     </row>
-    <row r="30" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1414,7 +1431,7 @@
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
     </row>
-    <row r="31" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1437,7 +1454,7 @@
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
     </row>
-    <row r="32" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1460,7 +1477,7 @@
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
     </row>
-    <row r="33" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1483,7 +1500,7 @@
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
     </row>
-    <row r="34" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1506,7 +1523,7 @@
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
     </row>
-    <row r="35" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1529,7 +1546,7 @@
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
     </row>
-    <row r="36" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1552,7 +1569,7 @@
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
     </row>
-    <row r="37" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1575,7 +1592,7 @@
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
     </row>
-    <row r="38" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1598,7 +1615,7 @@
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
     </row>
-    <row r="39" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1621,7 +1638,7 @@
       <c r="T39" s="3"/>
       <c r="U39" s="3"/>
     </row>
-    <row r="40" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1644,7 +1661,7 @@
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
     </row>
-    <row r="41" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1667,7 +1684,7 @@
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
     </row>
-    <row r="42" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1690,7 +1707,7 @@
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
     </row>
-    <row r="43" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1713,7 +1730,7 @@
       <c r="T43" s="3"/>
       <c r="U43" s="3"/>
     </row>
-    <row r="44" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1736,7 +1753,7 @@
       <c r="T44" s="3"/>
       <c r="U44" s="3"/>
     </row>
-    <row r="45" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1759,7 +1776,7 @@
       <c r="T45" s="3"/>
       <c r="U45" s="3"/>
     </row>
-    <row r="46" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1782,7 +1799,7 @@
       <c r="T46" s="3"/>
       <c r="U46" s="3"/>
     </row>
-    <row r="47" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1805,7 +1822,7 @@
       <c r="T47" s="3"/>
       <c r="U47" s="3"/>
     </row>
-    <row r="48" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -1828,7 +1845,7 @@
       <c r="T48" s="3"/>
       <c r="U48" s="3"/>
     </row>
-    <row r="49" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1851,7 +1868,7 @@
       <c r="T49" s="3"/>
       <c r="U49" s="3"/>
     </row>
-    <row r="50" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1874,7 +1891,7 @@
       <c r="T50" s="3"/>
       <c r="U50" s="3"/>
     </row>
-    <row r="51" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1897,7 +1914,7 @@
       <c r="T51" s="3"/>
       <c r="U51" s="3"/>
     </row>
-    <row r="52" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -1920,7 +1937,7 @@
       <c r="T52" s="3"/>
       <c r="U52" s="3"/>
     </row>
-    <row r="53" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1943,7 +1960,7 @@
       <c r="T53" s="3"/>
       <c r="U53" s="3"/>
     </row>
-    <row r="54" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1966,7 +1983,7 @@
       <c r="T54" s="3"/>
       <c r="U54" s="3"/>
     </row>
-    <row r="55" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1989,7 +2006,7 @@
       <c r="T55" s="3"/>
       <c r="U55" s="3"/>
     </row>
-    <row r="56" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -2012,7 +2029,7 @@
       <c r="T56" s="3"/>
       <c r="U56" s="3"/>
     </row>
-    <row r="57" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -2035,7 +2052,7 @@
       <c r="T57" s="3"/>
       <c r="U57" s="3"/>
     </row>
-    <row r="58" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -2058,7 +2075,7 @@
       <c r="T58" s="3"/>
       <c r="U58" s="3"/>
     </row>
-    <row r="59" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -2081,7 +2098,7 @@
       <c r="T59" s="3"/>
       <c r="U59" s="3"/>
     </row>
-    <row r="60" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -2104,7 +2121,7 @@
       <c r="T60" s="3"/>
       <c r="U60" s="3"/>
     </row>
-    <row r="61" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -2127,7 +2144,7 @@
       <c r="T61" s="3"/>
       <c r="U61" s="3"/>
     </row>
-    <row r="62" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -2150,7 +2167,7 @@
       <c r="T62" s="3"/>
       <c r="U62" s="3"/>
     </row>
-    <row r="63" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -2173,7 +2190,7 @@
       <c r="T63" s="3"/>
       <c r="U63" s="3"/>
     </row>
-    <row r="64" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -2196,7 +2213,7 @@
       <c r="T64" s="3"/>
       <c r="U64" s="3"/>
     </row>
-    <row r="65" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -2219,7 +2236,7 @@
       <c r="T65" s="3"/>
       <c r="U65" s="3"/>
     </row>
-    <row r="66" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -2242,7 +2259,7 @@
       <c r="T66" s="3"/>
       <c r="U66" s="3"/>
     </row>
-    <row r="67" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -2265,7 +2282,7 @@
       <c r="T67" s="3"/>
       <c r="U67" s="3"/>
     </row>
-    <row r="68" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -2288,7 +2305,7 @@
       <c r="T68" s="3"/>
       <c r="U68" s="3"/>
     </row>
-    <row r="69" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -2311,7 +2328,7 @@
       <c r="T69" s="3"/>
       <c r="U69" s="3"/>
     </row>
-    <row r="70" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -2334,7 +2351,7 @@
       <c r="T70" s="3"/>
       <c r="U70" s="3"/>
     </row>
-    <row r="71" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -2357,7 +2374,7 @@
       <c r="T71" s="3"/>
       <c r="U71" s="3"/>
     </row>
-    <row r="72" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -2380,7 +2397,7 @@
       <c r="T72" s="3"/>
       <c r="U72" s="3"/>
     </row>
-    <row r="73" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -2403,7 +2420,7 @@
       <c r="T73" s="3"/>
       <c r="U73" s="3"/>
     </row>
-    <row r="74" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -2426,7 +2443,7 @@
       <c r="T74" s="3"/>
       <c r="U74" s="3"/>
     </row>
-    <row r="75" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -2449,7 +2466,7 @@
       <c r="T75" s="3"/>
       <c r="U75" s="3"/>
     </row>
-    <row r="76" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -2472,7 +2489,7 @@
       <c r="T76" s="3"/>
       <c r="U76" s="3"/>
     </row>
-    <row r="77" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -2495,7 +2512,7 @@
       <c r="T77" s="3"/>
       <c r="U77" s="3"/>
     </row>
-    <row r="78" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -2518,7 +2535,7 @@
       <c r="T78" s="3"/>
       <c r="U78" s="3"/>
     </row>
-    <row r="79" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -2541,7 +2558,7 @@
       <c r="T79" s="3"/>
       <c r="U79" s="3"/>
     </row>
-    <row r="80" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -2564,7 +2581,7 @@
       <c r="T80" s="3"/>
       <c r="U80" s="3"/>
     </row>
-    <row r="81" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -2587,7 +2604,7 @@
       <c r="T81" s="3"/>
       <c r="U81" s="3"/>
     </row>
-    <row r="82" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -2610,7 +2627,7 @@
       <c r="T82" s="3"/>
       <c r="U82" s="3"/>
     </row>
-    <row r="83" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -2633,7 +2650,7 @@
       <c r="T83" s="3"/>
       <c r="U83" s="3"/>
     </row>
-    <row r="84" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -2656,7 +2673,7 @@
       <c r="T84" s="3"/>
       <c r="U84" s="3"/>
     </row>
-    <row r="85" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -2679,7 +2696,7 @@
       <c r="T85" s="3"/>
       <c r="U85" s="3"/>
     </row>
-    <row r="86" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -2702,7 +2719,7 @@
       <c r="T86" s="3"/>
       <c r="U86" s="3"/>
     </row>
-    <row r="87" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -2725,7 +2742,7 @@
       <c r="T87" s="3"/>
       <c r="U87" s="3"/>
     </row>
-    <row r="88" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -2748,7 +2765,7 @@
       <c r="T88" s="3"/>
       <c r="U88" s="3"/>
     </row>
-    <row r="89" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -2771,7 +2788,7 @@
       <c r="T89" s="3"/>
       <c r="U89" s="3"/>
     </row>
-    <row r="90" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -2794,7 +2811,7 @@
       <c r="T90" s="3"/>
       <c r="U90" s="3"/>
     </row>
-    <row r="91" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -2817,7 +2834,7 @@
       <c r="T91" s="3"/>
       <c r="U91" s="3"/>
     </row>
-    <row r="92" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -2840,7 +2857,7 @@
       <c r="T92" s="3"/>
       <c r="U92" s="3"/>
     </row>
-    <row r="93" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -2863,7 +2880,7 @@
       <c r="T93" s="3"/>
       <c r="U93" s="3"/>
     </row>
-    <row r="94" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -2886,7 +2903,7 @@
       <c r="T94" s="3"/>
       <c r="U94" s="3"/>
     </row>
-    <row r="95" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -2909,7 +2926,7 @@
       <c r="T95" s="3"/>
       <c r="U95" s="3"/>
     </row>
-    <row r="96" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -2932,7 +2949,7 @@
       <c r="T96" s="3"/>
       <c r="U96" s="3"/>
     </row>
-    <row r="97" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -2955,7 +2972,7 @@
       <c r="T97" s="3"/>
       <c r="U97" s="3"/>
     </row>
-    <row r="98" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -2978,7 +2995,7 @@
       <c r="T98" s="3"/>
       <c r="U98" s="3"/>
     </row>
-    <row r="99" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -3001,7 +3018,7 @@
       <c r="T99" s="3"/>
       <c r="U99" s="3"/>
     </row>
-    <row r="100" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -3024,7 +3041,7 @@
       <c r="T100" s="3"/>
       <c r="U100" s="3"/>
     </row>
-    <row r="101" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -3047,7 +3064,7 @@
       <c r="T101" s="3"/>
       <c r="U101" s="3"/>
     </row>
-    <row r="102" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -3070,7 +3087,7 @@
       <c r="T102" s="3"/>
       <c r="U102" s="3"/>
     </row>
-    <row r="103" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -3093,7 +3110,7 @@
       <c r="T103" s="3"/>
       <c r="U103" s="3"/>
     </row>
-    <row r="104" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -3116,7 +3133,7 @@
       <c r="T104" s="3"/>
       <c r="U104" s="3"/>
     </row>
-    <row r="105" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -3139,7 +3156,7 @@
       <c r="T105" s="3"/>
       <c r="U105" s="3"/>
     </row>
-    <row r="106" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -3162,7 +3179,7 @@
       <c r="T106" s="3"/>
       <c r="U106" s="3"/>
     </row>
-    <row r="107" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -3185,7 +3202,7 @@
       <c r="T107" s="3"/>
       <c r="U107" s="3"/>
     </row>
-    <row r="108" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -3208,7 +3225,7 @@
       <c r="T108" s="3"/>
       <c r="U108" s="3"/>
     </row>
-    <row r="109" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -3231,7 +3248,7 @@
       <c r="T109" s="3"/>
       <c r="U109" s="3"/>
     </row>
-    <row r="110" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -3254,7 +3271,7 @@
       <c r="T110" s="3"/>
       <c r="U110" s="3"/>
     </row>
-    <row r="111" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -3277,7 +3294,7 @@
       <c r="T111" s="3"/>
       <c r="U111" s="3"/>
     </row>
-    <row r="112" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -3300,7 +3317,7 @@
       <c r="T112" s="3"/>
       <c r="U112" s="3"/>
     </row>
-    <row r="113" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -3323,7 +3340,7 @@
       <c r="T113" s="3"/>
       <c r="U113" s="3"/>
     </row>
-    <row r="114" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -3346,7 +3363,7 @@
       <c r="T114" s="3"/>
       <c r="U114" s="3"/>
     </row>
-    <row r="115" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -3369,7 +3386,7 @@
       <c r="T115" s="3"/>
       <c r="U115" s="3"/>
     </row>
-    <row r="116" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -3392,7 +3409,7 @@
       <c r="T116" s="3"/>
       <c r="U116" s="3"/>
     </row>
-    <row r="117" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -3415,7 +3432,7 @@
       <c r="T117" s="3"/>
       <c r="U117" s="3"/>
     </row>
-    <row r="118" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -3438,7 +3455,7 @@
       <c r="T118" s="3"/>
       <c r="U118" s="3"/>
     </row>
-    <row r="119" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -3461,7 +3478,7 @@
       <c r="T119" s="3"/>
       <c r="U119" s="3"/>
     </row>
-    <row r="120" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -3484,7 +3501,7 @@
       <c r="T120" s="3"/>
       <c r="U120" s="3"/>
     </row>
-    <row r="121" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -3507,7 +3524,7 @@
       <c r="T121" s="3"/>
       <c r="U121" s="3"/>
     </row>
-    <row r="122" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -3530,7 +3547,7 @@
       <c r="T122" s="3"/>
       <c r="U122" s="3"/>
     </row>
-    <row r="123" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -3553,7 +3570,7 @@
       <c r="T123" s="3"/>
       <c r="U123" s="3"/>
     </row>
-    <row r="124" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -3576,7 +3593,7 @@
       <c r="T124" s="3"/>
       <c r="U124" s="3"/>
     </row>
-    <row r="125" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -3599,7 +3616,7 @@
       <c r="T125" s="3"/>
       <c r="U125" s="3"/>
     </row>
-    <row r="126" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -3622,7 +3639,7 @@
       <c r="T126" s="3"/>
       <c r="U126" s="3"/>
     </row>
-    <row r="127" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -3645,7 +3662,7 @@
       <c r="T127" s="3"/>
       <c r="U127" s="3"/>
     </row>
-    <row r="128" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -3668,7 +3685,7 @@
       <c r="T128" s="3"/>
       <c r="U128" s="3"/>
     </row>
-    <row r="129" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -3691,7 +3708,7 @@
       <c r="T129" s="3"/>
       <c r="U129" s="3"/>
     </row>
-    <row r="130" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -3714,7 +3731,7 @@
       <c r="T130" s="3"/>
       <c r="U130" s="3"/>
     </row>
-    <row r="131" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -3737,7 +3754,7 @@
       <c r="T131" s="3"/>
       <c r="U131" s="3"/>
     </row>
-    <row r="132" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -3760,7 +3777,7 @@
       <c r="T132" s="3"/>
       <c r="U132" s="3"/>
     </row>
-    <row r="133" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -3783,7 +3800,7 @@
       <c r="T133" s="3"/>
       <c r="U133" s="3"/>
     </row>
-    <row r="134" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -3806,7 +3823,7 @@
       <c r="T134" s="3"/>
       <c r="U134" s="3"/>
     </row>
-    <row r="135" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -3829,7 +3846,7 @@
       <c r="T135" s="3"/>
       <c r="U135" s="3"/>
     </row>
-    <row r="136" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
@@ -3852,7 +3869,7 @@
       <c r="T136" s="3"/>
       <c r="U136" s="3"/>
     </row>
-    <row r="137" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
@@ -3875,7 +3892,7 @@
       <c r="T137" s="3"/>
       <c r="U137" s="3"/>
     </row>
-    <row r="138" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
@@ -3898,7 +3915,7 @@
       <c r="T138" s="3"/>
       <c r="U138" s="3"/>
     </row>
-    <row r="139" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -3921,7 +3938,7 @@
       <c r="T139" s="3"/>
       <c r="U139" s="3"/>
     </row>
-    <row r="140" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -3944,7 +3961,7 @@
       <c r="T140" s="3"/>
       <c r="U140" s="3"/>
     </row>
-    <row r="141" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -3967,7 +3984,7 @@
       <c r="T141" s="3"/>
       <c r="U141" s="3"/>
     </row>
-    <row r="142" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -3990,7 +4007,7 @@
       <c r="T142" s="3"/>
       <c r="U142" s="3"/>
     </row>
-    <row r="143" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -4013,7 +4030,7 @@
       <c r="T143" s="3"/>
       <c r="U143" s="3"/>
     </row>
-    <row r="144" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
@@ -4036,7 +4053,7 @@
       <c r="T144" s="3"/>
       <c r="U144" s="3"/>
     </row>
-    <row r="145" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
@@ -4059,7 +4076,7 @@
       <c r="T145" s="3"/>
       <c r="U145" s="3"/>
     </row>
-    <row r="146" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -4082,7 +4099,7 @@
       <c r="T146" s="3"/>
       <c r="U146" s="3"/>
     </row>
-    <row r="147" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
@@ -4105,7 +4122,7 @@
       <c r="T147" s="3"/>
       <c r="U147" s="3"/>
     </row>
-    <row r="148" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
@@ -4128,7 +4145,7 @@
       <c r="T148" s="3"/>
       <c r="U148" s="3"/>
     </row>
-    <row r="149" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
@@ -4151,7 +4168,7 @@
       <c r="T149" s="3"/>
       <c r="U149" s="3"/>
     </row>
-    <row r="150" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
@@ -4174,7 +4191,7 @@
       <c r="T150" s="3"/>
       <c r="U150" s="3"/>
     </row>
-    <row r="151" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
@@ -4197,7 +4214,7 @@
       <c r="T151" s="3"/>
       <c r="U151" s="3"/>
     </row>
-    <row r="152" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
@@ -4220,7 +4237,7 @@
       <c r="T152" s="3"/>
       <c r="U152" s="3"/>
     </row>
-    <row r="153" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
@@ -4243,7 +4260,7 @@
       <c r="T153" s="3"/>
       <c r="U153" s="3"/>
     </row>
-    <row r="154" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
@@ -4266,7 +4283,7 @@
       <c r="T154" s="3"/>
       <c r="U154" s="3"/>
     </row>
-    <row r="155" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
@@ -4289,7 +4306,7 @@
       <c r="T155" s="3"/>
       <c r="U155" s="3"/>
     </row>
-    <row r="156" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
@@ -4312,7 +4329,7 @@
       <c r="T156" s="3"/>
       <c r="U156" s="3"/>
     </row>
-    <row r="157" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
@@ -4335,7 +4352,7 @@
       <c r="T157" s="3"/>
       <c r="U157" s="3"/>
     </row>
-    <row r="158" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
@@ -4358,7 +4375,7 @@
       <c r="T158" s="3"/>
       <c r="U158" s="3"/>
     </row>
-    <row r="159" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
@@ -4381,7 +4398,7 @@
       <c r="T159" s="3"/>
       <c r="U159" s="3"/>
     </row>
-    <row r="160" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
@@ -4404,7 +4421,7 @@
       <c r="T160" s="3"/>
       <c r="U160" s="3"/>
     </row>
-    <row r="161" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="3"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
@@ -4427,7 +4444,7 @@
       <c r="T161" s="3"/>
       <c r="U161" s="3"/>
     </row>
-    <row r="162" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -4450,7 +4467,7 @@
       <c r="T162" s="3"/>
       <c r="U162" s="3"/>
     </row>
-    <row r="163" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
@@ -4473,7 +4490,7 @@
       <c r="T163" s="3"/>
       <c r="U163" s="3"/>
     </row>
-    <row r="164" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
@@ -4496,7 +4513,7 @@
       <c r="T164" s="3"/>
       <c r="U164" s="3"/>
     </row>
-    <row r="165" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
@@ -4519,7 +4536,7 @@
       <c r="T165" s="3"/>
       <c r="U165" s="3"/>
     </row>
-    <row r="166" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
@@ -4542,7 +4559,7 @@
       <c r="T166" s="3"/>
       <c r="U166" s="3"/>
     </row>
-    <row r="167" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
@@ -4565,7 +4582,7 @@
       <c r="T167" s="3"/>
       <c r="U167" s="3"/>
     </row>
-    <row r="168" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
@@ -4588,7 +4605,7 @@
       <c r="T168" s="3"/>
       <c r="U168" s="3"/>
     </row>
-    <row r="169" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
@@ -4611,7 +4628,7 @@
       <c r="T169" s="3"/>
       <c r="U169" s="3"/>
     </row>
-    <row r="170" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
@@ -4634,7 +4651,7 @@
       <c r="T170" s="3"/>
       <c r="U170" s="3"/>
     </row>
-    <row r="171" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
@@ -4657,7 +4674,7 @@
       <c r="T171" s="3"/>
       <c r="U171" s="3"/>
     </row>
-    <row r="172" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
@@ -4680,7 +4697,7 @@
       <c r="T172" s="3"/>
       <c r="U172" s="3"/>
     </row>
-    <row r="173" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
@@ -4703,7 +4720,7 @@
       <c r="T173" s="3"/>
       <c r="U173" s="3"/>
     </row>
-    <row r="174" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
@@ -4726,7 +4743,7 @@
       <c r="T174" s="3"/>
       <c r="U174" s="3"/>
     </row>
-    <row r="175" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
@@ -4749,7 +4766,7 @@
       <c r="T175" s="3"/>
       <c r="U175" s="3"/>
     </row>
-    <row r="176" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
@@ -4772,7 +4789,7 @@
       <c r="T176" s="3"/>
       <c r="U176" s="3"/>
     </row>
-    <row r="177" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
@@ -4795,7 +4812,7 @@
       <c r="T177" s="3"/>
       <c r="U177" s="3"/>
     </row>
-    <row r="178" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
@@ -4818,7 +4835,7 @@
       <c r="T178" s="3"/>
       <c r="U178" s="3"/>
     </row>
-    <row r="179" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
@@ -4841,7 +4858,7 @@
       <c r="T179" s="3"/>
       <c r="U179" s="3"/>
     </row>
-    <row r="180" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
@@ -4864,7 +4881,7 @@
       <c r="T180" s="3"/>
       <c r="U180" s="3"/>
     </row>
-    <row r="181" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
@@ -4887,7 +4904,7 @@
       <c r="T181" s="3"/>
       <c r="U181" s="3"/>
     </row>
-    <row r="182" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
@@ -4910,7 +4927,7 @@
       <c r="T182" s="3"/>
       <c r="U182" s="3"/>
     </row>
-    <row r="183" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
@@ -4933,7 +4950,7 @@
       <c r="T183" s="3"/>
       <c r="U183" s="3"/>
     </row>
-    <row r="184" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
@@ -4956,7 +4973,7 @@
       <c r="T184" s="3"/>
       <c r="U184" s="3"/>
     </row>
-    <row r="185" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
@@ -4979,7 +4996,7 @@
       <c r="T185" s="3"/>
       <c r="U185" s="3"/>
     </row>
-    <row r="186" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
@@ -5002,7 +5019,7 @@
       <c r="T186" s="3"/>
       <c r="U186" s="3"/>
     </row>
-    <row r="187" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
@@ -5025,7 +5042,7 @@
       <c r="T187" s="3"/>
       <c r="U187" s="3"/>
     </row>
-    <row r="188" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
@@ -5048,7 +5065,7 @@
       <c r="T188" s="3"/>
       <c r="U188" s="3"/>
     </row>
-    <row r="189" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
@@ -5071,7 +5088,7 @@
       <c r="T189" s="3"/>
       <c r="U189" s="3"/>
     </row>
-    <row r="190" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
@@ -5094,7 +5111,7 @@
       <c r="T190" s="3"/>
       <c r="U190" s="3"/>
     </row>
-    <row r="191" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
@@ -5117,7 +5134,7 @@
       <c r="T191" s="3"/>
       <c r="U191" s="3"/>
     </row>
-    <row r="192" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
@@ -5140,7 +5157,7 @@
       <c r="T192" s="3"/>
       <c r="U192" s="3"/>
     </row>
-    <row r="193" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
@@ -5163,7 +5180,7 @@
       <c r="T193" s="3"/>
       <c r="U193" s="3"/>
     </row>
-    <row r="194" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
@@ -5186,7 +5203,7 @@
       <c r="T194" s="3"/>
       <c r="U194" s="3"/>
     </row>
-    <row r="195" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
@@ -5209,7 +5226,7 @@
       <c r="T195" s="3"/>
       <c r="U195" s="3"/>
     </row>
-    <row r="196" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
@@ -5232,7 +5249,7 @@
       <c r="T196" s="3"/>
       <c r="U196" s="3"/>
     </row>
-    <row r="197" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
@@ -5255,7 +5272,7 @@
       <c r="T197" s="3"/>
       <c r="U197" s="3"/>
     </row>
-    <row r="198" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
@@ -5278,7 +5295,7 @@
       <c r="T198" s="3"/>
       <c r="U198" s="3"/>
     </row>
-    <row r="199" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
@@ -5301,7 +5318,7 @@
       <c r="T199" s="3"/>
       <c r="U199" s="3"/>
     </row>
-    <row r="200" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -5325,33 +5342,12 @@
       <c r="U200" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="N10:N200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="N3:N200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="P10:P200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="P3:P200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="R10:R200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="R3:R200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T10:T200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T3:T200">
+  <dataValidations count="1">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T3:T200 R3:R200 P3:P200 N3:N200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>